<commit_message>
Agrega curvas de fabrica IntelliFlo VS+SVRS, WhisperFlo VST y WhisperFloXF
Incorpora al motor hidraulico las familias de bomba nuevas presentes en
la hoja de curvas Pentair (IntelliFlo VS+SVRS 3HP a 5 velocidades,
WhisperFlo VST 2HP a 4 velocidades, WhisperFloXF 3HP velocidad unica),
convertidas a m3/h y m c.a. El selector de origen de curva (CHK-074)
ahora las ofrece junto a las familias existentes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CURVAS CARÁCTERISTICAS BOMBAS CENTRÍFUGAS POR MODELO (PENTAIR).xlsx
+++ b/CURVAS CARÁCTERISTICAS BOMBAS CENTRÍFUGAS POR MODELO (PENTAIR).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/224e46dcc2f44639/Documentos/RES 929/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="8_{C6DE9229-EB19-4660-B4C4-E6956D4E10CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B10AE3F-18E4-41B2-9B84-5DD3269539D0}"/>
+  <xr:revisionPtr revIDLastSave="294" documentId="8_{C6DE9229-EB19-4660-B4C4-E6956D4E10CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4504A019-0E29-43CC-8767-E3F10F2BE875}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8374F0B3-CF22-49FB-9D25-798A4A8109C6}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="12360" windowHeight="15585" xr2:uid="{8374F0B3-CF22-49FB-9D25-798A4A8109C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="24">
   <si>
     <t>Total head (pie de agua)</t>
   </si>
@@ -78,6 +78,39 @@
   </si>
   <si>
     <t>SUPERFLO - 2,2HP VELOCIDAD 3 - 3450RPM</t>
+  </si>
+  <si>
+    <t>INTELLIFLO VS+SVRS VELOCIDAD 1 - 1100RPM</t>
+  </si>
+  <si>
+    <t>INTELLIFLO 3HP VS+SVRS VELOCIDAD 2 - 1500RPM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">caudal GPM - 60Hz </t>
+  </si>
+  <si>
+    <t>INTELLIFLO 3HP VS+SVRS VELOCIDAD 3 - 2350RPM</t>
+  </si>
+  <si>
+    <t>INTELLIFLO 3HP VS+SVRS VELOCIDAD 4 - 3110RPM</t>
+  </si>
+  <si>
+    <t>INTELLIFLO 3HP VS+SVRS VELOCIDAD MAX - 3450RPM</t>
+  </si>
+  <si>
+    <t>WHISPERFLOXF 3HP</t>
+  </si>
+  <si>
+    <t>WHISPERFLO VST 2HP - 1400RPM</t>
+  </si>
+  <si>
+    <t>WHISPERFLO VST 2HP - 2200RPM</t>
+  </si>
+  <si>
+    <t>WHISPERFLO VST 2HP - 3000RPM</t>
+  </si>
+  <si>
+    <t>WHISPERFLO VST 2HP - 3450RPM</t>
   </si>
 </sst>
 </file>
@@ -173,7 +206,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -181,11 +214,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -193,20 +232,11 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -223,6 +253,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -542,536 +576,982 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD19A7E-1381-451C-8D97-F082185B8189}">
-  <dimension ref="B1:E42"/>
+  <dimension ref="B1:I42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.21875" customWidth="1"/>
     <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="27.44140625" customWidth="1"/>
+    <col min="8" max="8" width="19.33203125" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="10"/>
+      <c r="D1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="6"/>
-    </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E1" s="8"/>
+      <c r="F1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="8"/>
+      <c r="H1" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="8"/>
+    </row>
+    <row r="2" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="7" t="s">
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B3" s="1">
         <v>0</v>
       </c>
       <c r="C3" s="1">
         <v>400</v>
       </c>
-      <c r="D3" s="7">
-        <v>0</v>
-      </c>
-      <c r="E3" s="7">
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3">
         <v>100</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="3">
+        <v>5</v>
+      </c>
+      <c r="G3" s="3">
+        <v>50</v>
+      </c>
+      <c r="H3" s="3">
+        <v>20</v>
+      </c>
+      <c r="I3" s="3">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B4" s="1">
         <v>20</v>
       </c>
       <c r="C4" s="1">
         <v>370</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="3">
         <v>20</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="3">
         <v>100</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F4" s="3">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3">
+        <v>40</v>
+      </c>
+      <c r="H4" s="3">
+        <v>30</v>
+      </c>
+      <c r="I4" s="3">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <v>40</v>
       </c>
       <c r="C5" s="1">
         <v>315</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="3">
         <v>40</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="3">
         <v>74</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="3">
+        <v>9</v>
+      </c>
+      <c r="G5" s="3">
+        <v>30</v>
+      </c>
+      <c r="H5" s="3">
+        <v>40</v>
+      </c>
+      <c r="I5" s="3">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B6" s="1">
         <v>60</v>
       </c>
       <c r="C6" s="1">
         <v>250</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="3">
         <v>50</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="3">
         <v>48</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="3">
+        <v>9.5</v>
+      </c>
+      <c r="G6" s="3">
+        <v>20</v>
+      </c>
+      <c r="H6" s="3">
+        <v>60</v>
+      </c>
+      <c r="I6" s="3">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <v>75</v>
       </c>
       <c r="C7" s="1">
         <v>100</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="3">
         <v>56</v>
       </c>
-      <c r="E7" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>10</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>90</v>
+      </c>
+      <c r="I7" s="3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B8" s="1">
         <v>80</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="6"/>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="3" t="s">
+      <c r="D8" s="7"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="3">
+        <v>100</v>
+      </c>
+      <c r="I8" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B9" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5" t="s">
+      <c r="C9" s="10"/>
+      <c r="D9" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="6"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E9" s="8"/>
+      <c r="F9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="8"/>
+      <c r="H9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="8"/>
+    </row>
+    <row r="10" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="7" t="s">
+      <c r="D10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B11" s="1">
         <v>0</v>
       </c>
       <c r="C11" s="1">
         <v>550</v>
       </c>
-      <c r="D11" s="7">
-        <v>0</v>
-      </c>
-      <c r="E11" s="7">
+      <c r="D11" s="3">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3">
         <v>70</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="3">
+        <v>7</v>
+      </c>
+      <c r="G11" s="3">
+        <v>70</v>
+      </c>
+      <c r="H11" s="3">
+        <v>3</v>
+      </c>
+      <c r="I11" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B12" s="1">
         <v>20</v>
       </c>
       <c r="C12" s="1">
         <v>510</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="3">
         <v>10</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="3">
         <v>70</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="3">
+        <v>10</v>
+      </c>
+      <c r="G12" s="3">
+        <v>62</v>
+      </c>
+      <c r="H12" s="3">
+        <v>5</v>
+      </c>
+      <c r="I12" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <v>40</v>
       </c>
       <c r="C13" s="1">
         <v>470</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="3">
         <v>20</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="3">
         <v>54</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="3">
+        <v>14</v>
+      </c>
+      <c r="G13" s="3">
+        <v>50</v>
+      </c>
+      <c r="H13" s="3">
+        <v>10</v>
+      </c>
+      <c r="I13" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B14" s="1">
         <v>60</v>
       </c>
       <c r="C14" s="1">
         <v>375</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="3">
         <v>28</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E14" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="3">
+        <v>18</v>
+      </c>
+      <c r="G14" s="3">
+        <v>20</v>
+      </c>
+      <c r="H14" s="3">
+        <v>12</v>
+      </c>
+      <c r="I14" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B15" s="1">
         <v>70</v>
       </c>
       <c r="C15" s="1">
         <v>300</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="3">
         <v>30</v>
       </c>
-      <c r="E15" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E15" s="3">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>19.8</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3">
+        <v>15</v>
+      </c>
+      <c r="I15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="1">
         <v>80</v>
       </c>
       <c r="C16" s="1">
         <v>0</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B17" s="3" t="s">
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16" s="8"/>
+    </row>
+    <row r="17" spans="2:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="5" t="s">
+      <c r="C17" s="10"/>
+      <c r="D17" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E17" s="6"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E17" s="8"/>
+      <c r="F17" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" s="8"/>
+      <c r="H17" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E18" s="7" t="s">
+      <c r="D18" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F18" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="3">
+        <v>12</v>
+      </c>
+      <c r="I18" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B19" s="1">
         <v>0</v>
       </c>
       <c r="C19" s="1">
         <v>600</v>
       </c>
-      <c r="D19" s="7">
-        <v>0</v>
-      </c>
-      <c r="E19" s="7">
+      <c r="D19" s="3">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3">
         <v>40</v>
       </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F19" s="3">
+        <v>18</v>
+      </c>
+      <c r="G19" s="3">
+        <v>115</v>
+      </c>
+      <c r="H19" s="3">
+        <v>15</v>
+      </c>
+      <c r="I19" s="3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B20" s="1">
         <v>20</v>
       </c>
       <c r="C20" s="1">
         <v>590</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="3">
         <v>5</v>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="3">
         <v>40</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F20" s="3">
+        <v>22</v>
+      </c>
+      <c r="G20" s="3">
+        <v>110</v>
+      </c>
+      <c r="H20" s="3">
+        <v>20</v>
+      </c>
+      <c r="I20" s="3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B21" s="1">
         <v>40</v>
       </c>
       <c r="C21" s="1">
         <v>530</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="3">
         <v>10</v>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="3">
         <v>25</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F21" s="3">
+        <v>26</v>
+      </c>
+      <c r="G21" s="3">
+        <v>100</v>
+      </c>
+      <c r="H21" s="3">
+        <v>30</v>
+      </c>
+      <c r="I21" s="3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B22" s="1">
         <v>60</v>
       </c>
       <c r="C22" s="1">
         <v>490</v>
       </c>
-      <c r="D22" s="7">
+      <c r="D22" s="3">
         <v>12</v>
       </c>
-      <c r="E22" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E22" s="3">
+        <v>0</v>
+      </c>
+      <c r="F22" s="3">
+        <v>39</v>
+      </c>
+      <c r="G22" s="3">
+        <v>60</v>
+      </c>
+      <c r="H22" s="3">
+        <v>32</v>
+      </c>
+      <c r="I22" s="3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="1">
         <v>70</v>
       </c>
       <c r="C23" s="2">
         <v>450</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E23" s="6"/>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E23" s="8"/>
+      <c r="F23" s="3">
+        <v>45</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3">
+        <v>35</v>
+      </c>
+      <c r="I23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B24" s="1">
         <v>80</v>
       </c>
       <c r="C24" s="2">
         <v>395</v>
       </c>
-      <c r="D24" s="7">
-        <v>0</v>
-      </c>
-      <c r="E24" s="7">
+      <c r="D24" s="3">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3">
         <v>110</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F24" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G24" s="8"/>
+      <c r="H24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" s="8"/>
+    </row>
+    <row r="25" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B25" s="1">
         <v>100</v>
       </c>
       <c r="C25" s="2">
         <v>200</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="3">
         <v>30</v>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="3">
         <v>110</v>
       </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F25" s="3">
+        <v>32</v>
+      </c>
+      <c r="G25" s="3">
+        <v>150</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B26" s="1">
         <v>105</v>
       </c>
       <c r="C26" s="2">
         <v>0</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="3">
         <v>40</v>
       </c>
-      <c r="E26" s="7">
+      <c r="E26" s="3">
         <v>97</v>
       </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B27" s="3" t="s">
+      <c r="F26" s="3">
+        <v>37</v>
+      </c>
+      <c r="G26" s="3">
+        <v>140</v>
+      </c>
+      <c r="H26" s="3">
+        <v>26</v>
+      </c>
+      <c r="I26" s="3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="7">
+      <c r="C27" s="10"/>
+      <c r="D27" s="3">
         <v>50</v>
       </c>
-      <c r="E27" s="7">
+      <c r="E27" s="3">
         <v>84</v>
       </c>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F27" s="3">
+        <v>57</v>
+      </c>
+      <c r="G27" s="3">
+        <v>100</v>
+      </c>
+      <c r="H27" s="3">
+        <v>30</v>
+      </c>
+      <c r="I27" s="3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B28" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="3">
         <v>74</v>
       </c>
-      <c r="E28" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E28" s="3">
+        <v>0</v>
+      </c>
+      <c r="F28" s="3">
+        <v>79</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3">
+        <v>40</v>
+      </c>
+      <c r="I28" s="3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="1">
         <v>0</v>
       </c>
       <c r="C29" s="1">
         <v>820</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E29" s="6"/>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E29" s="8"/>
+      <c r="F29" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" s="8"/>
+      <c r="H29" s="3">
+        <v>50</v>
+      </c>
+      <c r="I29" s="3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B30" s="1">
         <v>20</v>
       </c>
       <c r="C30" s="1">
         <v>800</v>
       </c>
-      <c r="D30" s="7">
-        <v>0</v>
-      </c>
-      <c r="E30" s="8">
+      <c r="D30" s="3">
+        <v>0</v>
+      </c>
+      <c r="E30" s="4">
         <v>89</v>
       </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F30" s="3">
+        <v>39</v>
+      </c>
+      <c r="G30" s="4">
+        <v>170</v>
+      </c>
+      <c r="H30" s="3">
+        <v>60</v>
+      </c>
+      <c r="I30" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B31" s="1">
         <v>40</v>
       </c>
       <c r="C31" s="1">
         <v>750</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="3">
         <v>20</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E31" s="4">
         <v>85</v>
       </c>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F31" s="3">
+        <v>60</v>
+      </c>
+      <c r="G31" s="4">
+        <v>140</v>
+      </c>
+      <c r="H31" s="3">
+        <v>65</v>
+      </c>
+      <c r="I31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B32" s="1">
         <v>60</v>
       </c>
       <c r="C32" s="1">
         <v>695</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D32" s="3">
         <v>40</v>
       </c>
-      <c r="E32" s="8">
+      <c r="E32" s="4">
         <v>66</v>
       </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F32" s="3">
+        <v>70</v>
+      </c>
+      <c r="G32" s="4">
+        <v>124</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I32" s="8"/>
+    </row>
+    <row r="33" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B33" s="1">
         <v>70</v>
       </c>
       <c r="C33" s="1">
         <v>650</v>
       </c>
-      <c r="D33" s="7">
+      <c r="D33" s="3">
         <v>50</v>
       </c>
-      <c r="E33" s="8">
+      <c r="E33" s="4">
         <v>54</v>
       </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F33" s="3">
+        <v>80</v>
+      </c>
+      <c r="G33" s="4">
+        <v>103</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B34" s="1">
         <v>80</v>
       </c>
       <c r="C34" s="1">
         <v>590</v>
       </c>
-      <c r="D34" s="7">
+      <c r="D34" s="3">
         <v>60</v>
       </c>
-      <c r="E34" s="8">
+      <c r="E34" s="4">
         <v>38</v>
       </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F34" s="3">
+        <v>90</v>
+      </c>
+      <c r="G34" s="4">
+        <v>74</v>
+      </c>
+      <c r="H34" s="3">
+        <v>38</v>
+      </c>
+      <c r="I34" s="3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B35" s="1">
         <v>100</v>
       </c>
       <c r="C35" s="1">
         <v>275</v>
       </c>
-      <c r="D35" s="7">
+      <c r="D35" s="3">
         <v>68</v>
       </c>
-      <c r="E35" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E35" s="4">
+        <v>0</v>
+      </c>
+      <c r="F35" s="3">
+        <v>97</v>
+      </c>
+      <c r="G35" s="4">
+        <v>0</v>
+      </c>
+      <c r="H35" s="3">
+        <v>45</v>
+      </c>
+      <c r="I35" s="3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="1">
         <v>112</v>
       </c>
       <c r="C36" s="1">
         <v>0</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E36" s="6"/>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D37" s="7">
-        <v>0</v>
-      </c>
-      <c r="E37" s="9">
+      <c r="E36" s="8"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="3">
+        <v>55</v>
+      </c>
+      <c r="I36" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D37" s="3">
+        <v>0</v>
+      </c>
+      <c r="E37" s="4">
         <v>72</v>
       </c>
-    </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D38" s="7">
+      <c r="F37" s="3"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="3">
+        <v>65</v>
+      </c>
+      <c r="I37" s="3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D38" s="3">
         <v>20</v>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="4">
         <v>65</v>
       </c>
-    </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D39" s="7">
+      <c r="F38" s="3"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="3">
+        <v>75</v>
+      </c>
+      <c r="I38" s="3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D39" s="3">
         <v>40</v>
       </c>
-      <c r="E39" s="9">
+      <c r="E39" s="4">
         <v>42</v>
       </c>
-    </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D40" s="7">
+      <c r="F39" s="3"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="3">
+        <v>87</v>
+      </c>
+      <c r="I39" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D40" s="3">
         <v>50</v>
       </c>
-      <c r="E40" s="9">
+      <c r="E40" s="4">
         <v>26</v>
       </c>
-    </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D41" s="7">
+      <c r="F40" s="3"/>
+      <c r="G40" s="4"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D41" s="3">
         <v>52</v>
       </c>
-      <c r="E41" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D42" s="10"/>
+      <c r="E41" s="4">
+        <v>0</v>
+      </c>
+      <c r="F41" s="3"/>
+      <c r="G41" s="4"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="23">
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F17:G17"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="D29:E29"/>

</xml_diff>